<commit_message>
Add marketplace link exports and harden network handling
</commit_message>
<xml_diff>
--- a/templates/client_mapping_template.xlsx
+++ b/templates/client_mapping_template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Клиент" sheetId="1" r:id="R8fef13a47ca04309"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Как использовать" sheetId="2" r:id="R1b5c1a4453ba482c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Клиент" sheetId="1" r:id="Rd2d8e4a7f2a341a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Как использовать" sheetId="2" r:id="R779f185ce5d5473e"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Improve supplier search image extraction
</commit_message>
<xml_diff>
--- a/templates/client_mapping_template.xlsx
+++ b/templates/client_mapping_template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Клиент" sheetId="1" r:id="Rd2d8e4a7f2a341a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Как использовать" sheetId="2" r:id="R779f185ce5d5473e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Клиент" sheetId="1" r:id="Ra9a4f811ca1f41bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Как использовать" sheetId="2" r:id="R819228ce171844e7"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>